<commit_message>
added templates needs testing esp obo
</commit_message>
<xml_diff>
--- a/docassemble/PowerOfAttorneyProperty/data/sources/poa_property_es.xlsx
+++ b/docassemble/PowerOfAttorneyProperty/data/sources/poa_property_es.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\local-DA-easyforms-dev\sources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1B12DC0-F368-4826-A16B-EA88C483B0D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9495667D-5045-4CC4-97C3-7A3E412DCFAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11942,94 +11942,6 @@
     <t>59f97fe5b9ca4961f0d468f1bb28401e</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">They can create a Power of Attorney Revocation to end a Power of Attorney.
-To make a Power of Attorney Revocation, use ILAO's </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[**Power of Attorney Revocation Easy Form**]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>https://www.illinoislegalaid.org/legal-information/power-attorney-revocation</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">).
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Pueden crear una Revocación de Poder para terminar un poder.
-Para hacer una Revocación de Poder, use el </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[Power of Attorney Revocation Easy Form]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> de ILAO.</t>
-    </r>
-  </si>
-  <si>
     <t>10b1c7c68ea5ce648fe1552ca8cafebc</t>
   </si>
   <si>
@@ -26198,6 +26110,38 @@
       </rPr>
       <t>% endif</t>
     </r>
+  </si>
+  <si>
+    <r>
+      <t>They can create a Power of Attorney Revocation to end a Power of Attorney.
+To make a Power of Attorney Revocation, use ILAO's [**Power of Attorney Revocation Easy Form**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://www.illinoislegalaid.org/legal-information/power-attorney-revocation</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">).
+</t>
+    </r>
+  </si>
+  <si>
+    <t>Pueden crear una Revocación de Poder para terminar un poder.
+Para hacer una Revocación de Poder, use el [**Formulario Fácil de Revocación de Poder Notarial**](https://es.illinoislegalaid.org/legal-information/power-attorney-revocation) de ILAO].</t>
   </si>
 </sst>
 </file>
@@ -26673,7 +26617,7 @@
         <v>13</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>782</v>
+        <v>780</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="403.2">
@@ -26687,7 +26631,7 @@
         <v>1</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>845</v>
+        <v>843</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>11</v>
@@ -26696,10 +26640,10 @@
         <v>12</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>846</v>
+        <v>844</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>847</v>
+        <v>845</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="187.2">
@@ -26725,7 +26669,7 @@
         <v>16</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="28.8">
@@ -26751,7 +26695,7 @@
         <v>19</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="302.39999999999998">
@@ -26777,7 +26721,7 @@
         <v>21</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>848</v>
+        <v>846</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -26803,7 +26747,7 @@
         <v>24</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>745</v>
+        <v>743</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="72">
@@ -26829,7 +26773,7 @@
         <v>26</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>785</v>
+        <v>783</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -26855,7 +26799,7 @@
         <v>28</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="43.2">
@@ -26881,7 +26825,7 @@
         <v>30</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>786</v>
+        <v>784</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="28.8">
@@ -26933,7 +26877,7 @@
         <v>35</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>787</v>
+        <v>785</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="43.2">
@@ -26959,7 +26903,7 @@
         <v>38</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>788</v>
+        <v>786</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="43.2">
@@ -26985,7 +26929,7 @@
         <v>40</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>789</v>
+        <v>787</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="86.4">
@@ -27011,7 +26955,7 @@
         <v>43</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>851</v>
+        <v>849</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="115.2">
@@ -27037,7 +26981,7 @@
         <v>46</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>849</v>
+        <v>847</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="28.8">
@@ -27089,7 +27033,7 @@
         <v>52</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>790</v>
+        <v>788</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="273.60000000000002">
@@ -27115,7 +27059,7 @@
         <v>54</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>850</v>
+        <v>848</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="28.8">
@@ -27141,7 +27085,7 @@
         <v>57</v>
       </c>
       <c r="H20" t="s">
-        <v>791</v>
+        <v>789</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="129.6">
@@ -27167,7 +27111,7 @@
         <v>59</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>792</v>
+        <v>790</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -27193,7 +27137,7 @@
         <v>62</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>793</v>
+        <v>791</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="43.2">
@@ -27219,7 +27163,7 @@
         <v>64</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>794</v>
+        <v>792</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="72">
@@ -27245,7 +27189,7 @@
         <v>66</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>795</v>
+        <v>793</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="28.8">
@@ -27271,7 +27215,7 @@
         <v>68</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>796</v>
+        <v>794</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="57.6">
@@ -27297,7 +27241,7 @@
         <v>70</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>856</v>
+        <v>854</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -27323,7 +27267,7 @@
         <v>72</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>797</v>
+        <v>795</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -27349,7 +27293,7 @@
         <v>74</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>798</v>
+        <v>796</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="28.8">
@@ -27375,7 +27319,7 @@
         <v>77</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>799</v>
+        <v>797</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="259.2">
@@ -27401,7 +27345,7 @@
         <v>79</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>800</v>
+        <v>798</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="86.4">
@@ -27427,7 +27371,7 @@
         <v>82</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>801</v>
+        <v>799</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="403.2">
@@ -27453,7 +27397,7 @@
         <v>84</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>802</v>
+        <v>800</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -27479,7 +27423,7 @@
         <v>86</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>803</v>
+        <v>801</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -27505,7 +27449,7 @@
         <v>88</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>804</v>
+        <v>802</v>
       </c>
     </row>
     <row r="35" spans="1:8">
@@ -27531,7 +27475,7 @@
         <v>90</v>
       </c>
       <c r="H35" s="4" t="s">
-        <v>805</v>
+        <v>803</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -27557,7 +27501,7 @@
         <v>92</v>
       </c>
       <c r="H36" s="5" t="s">
-        <v>806</v>
+        <v>804</v>
       </c>
     </row>
     <row r="37" spans="1:8">
@@ -27609,7 +27553,7 @@
         <v>97</v>
       </c>
       <c r="H38" s="4" t="s">
-        <v>807</v>
+        <v>805</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="115.2">
@@ -27635,7 +27579,7 @@
         <v>100</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>808</v>
+        <v>806</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="28.8">
@@ -27661,7 +27605,7 @@
         <v>102</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="28.8">
@@ -27687,7 +27631,7 @@
         <v>105</v>
       </c>
       <c r="H41" s="3" t="s">
-        <v>810</v>
+        <v>808</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="86.4">
@@ -27713,7 +27657,7 @@
         <v>108</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>857</v>
+        <v>855</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="28.8">
@@ -27739,7 +27683,7 @@
         <v>111</v>
       </c>
       <c r="H43" s="4" t="s">
-        <v>858</v>
+        <v>856</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="144">
@@ -27791,7 +27735,7 @@
         <v>117</v>
       </c>
       <c r="H45" s="3" t="s">
-        <v>811</v>
+        <v>809</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="86.4">
@@ -27817,7 +27761,7 @@
         <v>120</v>
       </c>
       <c r="H46" s="3" t="s">
-        <v>812</v>
+        <v>810</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="86.4">
@@ -27843,7 +27787,7 @@
         <v>123</v>
       </c>
       <c r="H47" s="3" t="s">
-        <v>813</v>
+        <v>811</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="345.6">
@@ -27869,7 +27813,7 @@
         <v>125</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>814</v>
+        <v>812</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="28.8">
@@ -27895,7 +27839,7 @@
         <v>128</v>
       </c>
       <c r="H49" s="3" t="s">
-        <v>815</v>
+        <v>813</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="28.8">
@@ -27947,7 +27891,7 @@
         <v>133</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>816</v>
+        <v>814</v>
       </c>
     </row>
     <row r="52" spans="1:8" ht="43.2">
@@ -27973,7 +27917,7 @@
         <v>135</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>817</v>
+        <v>815</v>
       </c>
     </row>
     <row r="53" spans="1:8">
@@ -27999,7 +27943,7 @@
         <v>137</v>
       </c>
       <c r="H53" t="s">
-        <v>860</v>
+        <v>858</v>
       </c>
     </row>
     <row r="54" spans="1:8">
@@ -28025,7 +27969,7 @@
         <v>139</v>
       </c>
       <c r="H54" t="s">
-        <v>861</v>
+        <v>859</v>
       </c>
     </row>
     <row r="55" spans="1:8" ht="129.6">
@@ -28051,7 +27995,7 @@
         <v>142</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>852</v>
+        <v>850</v>
       </c>
     </row>
     <row r="56" spans="1:8" ht="28.8">
@@ -28077,7 +28021,7 @@
         <v>144</v>
       </c>
       <c r="H56" s="4" t="s">
-        <v>859</v>
+        <v>857</v>
       </c>
     </row>
     <row r="57" spans="1:8" ht="28.8">
@@ -28129,7 +28073,7 @@
         <v>150</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>818</v>
+        <v>816</v>
       </c>
     </row>
     <row r="59" spans="1:8" ht="115.2">
@@ -28155,7 +28099,7 @@
         <v>153</v>
       </c>
       <c r="H59" s="5" t="s">
-        <v>862</v>
+        <v>860</v>
       </c>
     </row>
     <row r="60" spans="1:8" ht="28.8">
@@ -28207,7 +28151,7 @@
         <v>159</v>
       </c>
       <c r="H61" s="3" t="s">
-        <v>819</v>
+        <v>817</v>
       </c>
     </row>
     <row r="62" spans="1:8" ht="244.8">
@@ -28233,7 +28177,7 @@
         <v>161</v>
       </c>
       <c r="H62" s="3" t="s">
-        <v>820</v>
+        <v>818</v>
       </c>
     </row>
     <row r="63" spans="1:8">
@@ -28259,7 +28203,7 @@
         <v>163</v>
       </c>
       <c r="H63" s="3" t="s">
-        <v>821</v>
+        <v>819</v>
       </c>
     </row>
     <row r="64" spans="1:8">
@@ -28285,7 +28229,7 @@
         <v>165</v>
       </c>
       <c r="H64" s="4" t="s">
-        <v>822</v>
+        <v>820</v>
       </c>
     </row>
     <row r="65" spans="1:8" ht="43.2">
@@ -28337,7 +28281,7 @@
         <v>170</v>
       </c>
       <c r="H66" s="4" t="s">
-        <v>823</v>
+        <v>821</v>
       </c>
     </row>
     <row r="67" spans="1:8" ht="43.2">
@@ -28363,7 +28307,7 @@
         <v>172</v>
       </c>
       <c r="H67" s="4" t="s">
-        <v>863</v>
+        <v>861</v>
       </c>
     </row>
     <row r="68" spans="1:8">
@@ -28415,7 +28359,7 @@
         <v>177</v>
       </c>
       <c r="H69" s="4" t="s">
-        <v>824</v>
+        <v>822</v>
       </c>
     </row>
     <row r="70" spans="1:8">
@@ -28441,7 +28385,7 @@
         <v>179</v>
       </c>
       <c r="H70" s="4" t="s">
-        <v>825</v>
+        <v>823</v>
       </c>
     </row>
     <row r="71" spans="1:8" ht="72">
@@ -28467,7 +28411,7 @@
         <v>181</v>
       </c>
       <c r="H71" s="4" t="s">
-        <v>826</v>
+        <v>824</v>
       </c>
     </row>
     <row r="72" spans="1:8">
@@ -28493,7 +28437,7 @@
         <v>183</v>
       </c>
       <c r="H72" s="4" t="s">
-        <v>827</v>
+        <v>825</v>
       </c>
     </row>
     <row r="73" spans="1:8" ht="43.2">
@@ -28519,7 +28463,7 @@
         <v>185</v>
       </c>
       <c r="H73" s="4" t="s">
-        <v>828</v>
+        <v>826</v>
       </c>
     </row>
     <row r="74" spans="1:8">
@@ -28571,7 +28515,7 @@
         <v>190</v>
       </c>
       <c r="H75" s="4" t="s">
-        <v>830</v>
+        <v>828</v>
       </c>
     </row>
     <row r="76" spans="1:8">
@@ -28597,7 +28541,7 @@
         <v>192</v>
       </c>
       <c r="H76" s="4" t="s">
-        <v>829</v>
+        <v>827</v>
       </c>
     </row>
     <row r="77" spans="1:8" ht="43.2">
@@ -28623,7 +28567,7 @@
         <v>194</v>
       </c>
       <c r="H77" s="4" t="s">
-        <v>831</v>
+        <v>829</v>
       </c>
     </row>
     <row r="78" spans="1:8">
@@ -28649,7 +28593,7 @@
         <v>196</v>
       </c>
       <c r="H78" s="4" t="s">
-        <v>832</v>
+        <v>830</v>
       </c>
     </row>
     <row r="79" spans="1:8" ht="57.6">
@@ -28675,7 +28619,7 @@
         <v>198</v>
       </c>
       <c r="H79" s="4" t="s">
-        <v>833</v>
+        <v>831</v>
       </c>
     </row>
     <row r="80" spans="1:8">
@@ -28727,7 +28671,7 @@
         <v>203</v>
       </c>
       <c r="H81" s="4" t="s">
-        <v>834</v>
+        <v>832</v>
       </c>
     </row>
     <row r="82" spans="1:8">
@@ -28779,7 +28723,7 @@
         <v>208</v>
       </c>
       <c r="H83" s="4" t="s">
-        <v>835</v>
+        <v>833</v>
       </c>
     </row>
     <row r="84" spans="1:8">
@@ -28831,7 +28775,7 @@
         <v>213</v>
       </c>
       <c r="H85" s="4" t="s">
-        <v>836</v>
+        <v>834</v>
       </c>
     </row>
     <row r="86" spans="1:8">
@@ -28883,7 +28827,7 @@
         <v>218</v>
       </c>
       <c r="H87" s="4" t="s">
-        <v>837</v>
+        <v>835</v>
       </c>
     </row>
     <row r="88" spans="1:8">
@@ -28935,7 +28879,7 @@
         <v>223</v>
       </c>
       <c r="H89" s="4" t="s">
-        <v>839</v>
+        <v>837</v>
       </c>
     </row>
     <row r="90" spans="1:8">
@@ -28961,7 +28905,7 @@
         <v>225</v>
       </c>
       <c r="H90" s="4" t="s">
-        <v>838</v>
+        <v>836</v>
       </c>
     </row>
     <row r="91" spans="1:8" ht="43.2">
@@ -28987,7 +28931,7 @@
         <v>227</v>
       </c>
       <c r="H91" s="4" t="s">
-        <v>840</v>
+        <v>838</v>
       </c>
     </row>
     <row r="92" spans="1:8">
@@ -29039,7 +28983,7 @@
         <v>232</v>
       </c>
       <c r="H93" s="4" t="s">
-        <v>841</v>
+        <v>839</v>
       </c>
     </row>
     <row r="94" spans="1:8">
@@ -29091,7 +29035,7 @@
         <v>238</v>
       </c>
       <c r="H95" s="3" t="s">
-        <v>842</v>
+        <v>840</v>
       </c>
     </row>
     <row r="96" spans="1:8" ht="100.8">
@@ -29117,7 +29061,7 @@
         <v>241</v>
       </c>
       <c r="H96" s="3" t="s">
-        <v>843</v>
+        <v>841</v>
       </c>
     </row>
     <row r="97" spans="1:8" ht="115.2">
@@ -29143,7 +29087,7 @@
         <v>244</v>
       </c>
       <c r="H97" s="3" t="s">
-        <v>844</v>
+        <v>842</v>
       </c>
     </row>
     <row r="98" spans="1:8" ht="259.2">
@@ -29169,7 +29113,7 @@
         <v>246</v>
       </c>
       <c r="H98" s="3" t="s">
-        <v>853</v>
+        <v>851</v>
       </c>
     </row>
     <row r="99" spans="1:8" ht="28.8">
@@ -29221,7 +29165,7 @@
         <v>252</v>
       </c>
       <c r="H100" s="3" t="s">
-        <v>854</v>
+        <v>852</v>
       </c>
     </row>
     <row r="101" spans="1:8" ht="86.4">
@@ -30703,7 +30647,7 @@
         <v>433</v>
       </c>
       <c r="H157" s="4" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
     </row>
     <row r="158" spans="1:8">
@@ -30807,7 +30751,7 @@
         <v>444</v>
       </c>
       <c r="H161" s="3" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
     </row>
     <row r="162" spans="1:8" ht="86.4">
@@ -31015,7 +30959,7 @@
         <v>471</v>
       </c>
       <c r="H169" s="3" t="s">
-        <v>866</v>
+        <v>864</v>
       </c>
     </row>
     <row r="170" spans="1:8" ht="28.8">
@@ -31119,7 +31063,7 @@
         <v>484</v>
       </c>
       <c r="H173" s="5" t="s">
-        <v>869</v>
+        <v>867</v>
       </c>
     </row>
     <row r="174" spans="1:8" ht="28.8">
@@ -31145,7 +31089,7 @@
         <v>486</v>
       </c>
       <c r="H174" s="4" t="s">
-        <v>868</v>
+        <v>866</v>
       </c>
     </row>
     <row r="175" spans="1:8">
@@ -31301,7 +31245,7 @@
         <v>504</v>
       </c>
       <c r="H180" s="3" t="s">
-        <v>867</v>
+        <v>865</v>
       </c>
     </row>
     <row r="181" spans="1:8">
@@ -31535,7 +31479,7 @@
         <v>531</v>
       </c>
       <c r="H189" s="4" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
     </row>
     <row r="190" spans="1:8" ht="115.2">
@@ -31561,7 +31505,7 @@
         <v>534</v>
       </c>
       <c r="H190" s="3" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
     </row>
     <row r="191" spans="1:8" ht="28.8">
@@ -31636,10 +31580,10 @@
         <v>12</v>
       </c>
       <c r="G193" s="3" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
       <c r="H193" s="3" t="s">
-        <v>873</v>
+        <v>871</v>
       </c>
     </row>
     <row r="194" spans="1:8" ht="86.4">
@@ -31662,10 +31606,10 @@
         <v>12</v>
       </c>
       <c r="G194" s="3" t="s">
-        <v>545</v>
-      </c>
-      <c r="H194" s="3" t="s">
-        <v>546</v>
+        <v>872</v>
+      </c>
+      <c r="H194" s="4" t="s">
+        <v>873</v>
       </c>
     </row>
     <row r="195" spans="1:8" ht="28.8">
@@ -31679,7 +31623,7 @@
         <v>1</v>
       </c>
       <c r="D195" s="2" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="E195" s="2" t="s">
         <v>11</v>
@@ -31688,10 +31632,10 @@
         <v>12</v>
       </c>
       <c r="G195" s="3" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="H195" s="4" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
     </row>
     <row r="196" spans="1:8" ht="86.4">
@@ -31699,13 +31643,13 @@
         <v>8</v>
       </c>
       <c r="B196" s="2" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="C196" s="2">
         <v>0</v>
       </c>
       <c r="D196" s="2" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="E196" s="2" t="s">
         <v>11</v>
@@ -31714,10 +31658,10 @@
         <v>12</v>
       </c>
       <c r="G196" s="3" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="H196" s="3" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
     </row>
     <row r="197" spans="1:8" ht="201.6">
@@ -31725,13 +31669,13 @@
         <v>8</v>
       </c>
       <c r="B197" s="2" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="C197" s="2">
         <v>1</v>
       </c>
       <c r="D197" s="2" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="E197" s="2" t="s">
         <v>11</v>
@@ -31740,10 +31684,10 @@
         <v>12</v>
       </c>
       <c r="G197" s="3" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="H197" s="3" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="198" spans="1:8" ht="28.8">
@@ -31751,13 +31695,13 @@
         <v>8</v>
       </c>
       <c r="B198" s="2" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="C198" s="2">
         <v>2</v>
       </c>
       <c r="D198" s="2" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="E198" s="2" t="s">
         <v>11</v>
@@ -31766,10 +31710,10 @@
         <v>12</v>
       </c>
       <c r="G198" s="3" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="H198" s="3" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
     </row>
     <row r="199" spans="1:8">
@@ -31777,13 +31721,13 @@
         <v>8</v>
       </c>
       <c r="B199" s="2" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="C199" s="2">
         <v>3</v>
       </c>
       <c r="D199" s="2" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="E199" s="2" t="s">
         <v>11</v>
@@ -31792,10 +31736,10 @@
         <v>12</v>
       </c>
       <c r="G199" s="3" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="H199" s="3" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
     </row>
     <row r="200" spans="1:8" ht="100.8">
@@ -31803,13 +31747,13 @@
         <v>8</v>
       </c>
       <c r="B200" s="2" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="C200" s="2">
         <v>4</v>
       </c>
       <c r="D200" s="2" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="E200" s="2" t="s">
         <v>11</v>
@@ -31818,10 +31762,10 @@
         <v>12</v>
       </c>
       <c r="G200" s="3" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="H200" s="4" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
     </row>
     <row r="201" spans="1:8" ht="28.8">
@@ -31829,13 +31773,13 @@
         <v>8</v>
       </c>
       <c r="B201" s="2" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="C201" s="2">
         <v>5</v>
       </c>
       <c r="D201" s="2" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="E201" s="2" t="s">
         <v>11</v>
@@ -31844,10 +31788,10 @@
         <v>12</v>
       </c>
       <c r="G201" s="3" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="H201" s="3" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
     </row>
     <row r="202" spans="1:8">
@@ -31855,13 +31799,13 @@
         <v>8</v>
       </c>
       <c r="B202" s="2" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="C202" s="2">
         <v>6</v>
       </c>
       <c r="D202" s="2" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="E202" s="2" t="s">
         <v>11</v>
@@ -31870,10 +31814,10 @@
         <v>12</v>
       </c>
       <c r="G202" s="3" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="H202" s="4" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
     </row>
     <row r="203" spans="1:8">
@@ -31881,13 +31825,13 @@
         <v>8</v>
       </c>
       <c r="B203" s="2" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="C203" s="2">
         <v>7</v>
       </c>
       <c r="D203" s="2" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="E203" s="2" t="s">
         <v>11</v>
@@ -31896,10 +31840,10 @@
         <v>12</v>
       </c>
       <c r="G203" s="3" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="H203" s="4" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
     </row>
     <row r="204" spans="1:8" ht="100.8">
@@ -31907,13 +31851,13 @@
         <v>8</v>
       </c>
       <c r="B204" s="2" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="C204" s="2">
         <v>0</v>
       </c>
       <c r="D204" s="2" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="E204" s="2" t="s">
         <v>11</v>
@@ -31922,10 +31866,10 @@
         <v>12</v>
       </c>
       <c r="G204" s="3" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="H204" s="3" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
     </row>
     <row r="205" spans="1:8" ht="244.8">
@@ -31933,13 +31877,13 @@
         <v>8</v>
       </c>
       <c r="B205" s="2" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="C205" s="2">
         <v>1</v>
       </c>
       <c r="D205" s="2" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="E205" s="2" t="s">
         <v>11</v>
@@ -31948,10 +31892,10 @@
         <v>12</v>
       </c>
       <c r="G205" s="3" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="H205" s="3" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
     </row>
     <row r="206" spans="1:8" ht="28.8">
@@ -31959,13 +31903,13 @@
         <v>8</v>
       </c>
       <c r="B206" s="2" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="C206" s="2">
         <v>0</v>
       </c>
       <c r="D206" s="2" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="E206" s="2" t="s">
         <v>11</v>
@@ -31974,10 +31918,10 @@
         <v>12</v>
       </c>
       <c r="G206" s="3" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="H206" s="4" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
     </row>
     <row r="207" spans="1:8" ht="43.2">
@@ -31985,13 +31929,13 @@
         <v>8</v>
       </c>
       <c r="B207" s="2" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="C207" s="2">
         <v>1</v>
       </c>
       <c r="D207" s="2" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="E207" s="2" t="s">
         <v>11</v>
@@ -32000,10 +31944,10 @@
         <v>12</v>
       </c>
       <c r="G207" s="3" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="H207" s="3" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
     </row>
     <row r="208" spans="1:8" ht="28.8">
@@ -32011,13 +31955,13 @@
         <v>8</v>
       </c>
       <c r="B208" s="2" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="C208" s="2">
         <v>0</v>
       </c>
       <c r="D208" s="2" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="E208" s="2" t="s">
         <v>11</v>
@@ -32026,10 +31970,10 @@
         <v>12</v>
       </c>
       <c r="G208" s="3" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="H208" s="4" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
     </row>
     <row r="209" spans="1:8" ht="28.8">
@@ -32037,13 +31981,13 @@
         <v>8</v>
       </c>
       <c r="B209" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="C209" s="2">
         <v>0</v>
       </c>
       <c r="D209" s="2" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="E209" s="2" t="s">
         <v>11</v>
@@ -32052,10 +31996,10 @@
         <v>12</v>
       </c>
       <c r="G209" s="3" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="H209" s="4" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
     </row>
     <row r="210" spans="1:8" ht="28.8">
@@ -32063,13 +32007,13 @@
         <v>8</v>
       </c>
       <c r="B210" s="2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="C210" s="2">
         <v>1</v>
       </c>
       <c r="D210" s="2" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="E210" s="2" t="s">
         <v>11</v>
@@ -32078,10 +32022,10 @@
         <v>12</v>
       </c>
       <c r="G210" s="3" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="H210" s="4" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
     </row>
     <row r="211" spans="1:8" ht="28.8">
@@ -32089,13 +32033,13 @@
         <v>8</v>
       </c>
       <c r="B211" s="2" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="C211" s="2">
         <v>0</v>
       </c>
       <c r="D211" s="2" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="E211" s="2" t="s">
         <v>11</v>
@@ -32104,10 +32048,10 @@
         <v>12</v>
       </c>
       <c r="G211" s="3" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="H211" s="4" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
     </row>
     <row r="212" spans="1:8" ht="409.6">
@@ -32115,13 +32059,13 @@
         <v>8</v>
       </c>
       <c r="B212" s="2" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="C212" s="2">
         <v>1</v>
       </c>
       <c r="D212" s="2" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="E212" s="2" t="s">
         <v>11</v>
@@ -32130,10 +32074,10 @@
         <v>12</v>
       </c>
       <c r="G212" s="3" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="H212" s="3" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
     </row>
     <row r="213" spans="1:8" ht="86.4">
@@ -32141,13 +32085,13 @@
         <v>8</v>
       </c>
       <c r="B213" s="2" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="C213" s="2">
         <v>0</v>
       </c>
       <c r="D213" s="2" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="E213" s="2" t="s">
         <v>11</v>
@@ -32156,10 +32100,10 @@
         <v>12</v>
       </c>
       <c r="G213" s="3" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="H213" s="4" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
     </row>
     <row r="214" spans="1:8" ht="86.4">
@@ -32167,13 +32111,13 @@
         <v>8</v>
       </c>
       <c r="B214" s="2" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="C214" s="2">
         <v>1</v>
       </c>
       <c r="D214" s="2" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="E214" s="2" t="s">
         <v>11</v>
@@ -32182,10 +32126,10 @@
         <v>12</v>
       </c>
       <c r="G214" s="3" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="H214" s="3" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
     </row>
     <row r="215" spans="1:8" ht="28.8">
@@ -32193,13 +32137,13 @@
         <v>8</v>
       </c>
       <c r="B215" s="2" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="C215" s="2">
         <v>0</v>
       </c>
       <c r="D215" s="2" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="E215" s="2" t="s">
         <v>11</v>
@@ -32208,10 +32152,10 @@
         <v>12</v>
       </c>
       <c r="G215" s="3" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="H215" s="4" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
     </row>
     <row r="216" spans="1:8" ht="403.2">
@@ -32219,13 +32163,13 @@
         <v>8</v>
       </c>
       <c r="B216" s="2" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="C216" s="2">
         <v>1</v>
       </c>
       <c r="D216" s="2" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="E216" s="2" t="s">
         <v>11</v>
@@ -32234,10 +32178,10 @@
         <v>12</v>
       </c>
       <c r="G216" s="3" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="H216" s="3" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
     </row>
     <row r="217" spans="1:8" ht="187.2">
@@ -32245,13 +32189,13 @@
         <v>8</v>
       </c>
       <c r="B217" s="2" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="C217" s="2">
         <v>2</v>
       </c>
       <c r="D217" s="2" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="E217" s="2" t="s">
         <v>11</v>
@@ -32260,10 +32204,10 @@
         <v>12</v>
       </c>
       <c r="G217" s="3" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="H217" s="3" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
     </row>
     <row r="218" spans="1:8" ht="86.4">
@@ -32271,13 +32215,13 @@
         <v>8</v>
       </c>
       <c r="B218" s="2" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="C218" s="2">
         <v>0</v>
       </c>
       <c r="D218" s="2" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="E218" s="2" t="s">
         <v>11</v>
@@ -32286,10 +32230,10 @@
         <v>12</v>
       </c>
       <c r="G218" s="3" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="H218" s="3" t="s">
-        <v>855</v>
+        <v>853</v>
       </c>
     </row>
     <row r="219" spans="1:8">
@@ -32297,13 +32241,13 @@
         <v>8</v>
       </c>
       <c r="B219" s="2" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="C219" s="2">
         <v>1</v>
       </c>
       <c r="D219" s="2" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="E219" s="2" t="s">
         <v>11</v>
@@ -32315,7 +32259,7 @@
         <v>22</v>
       </c>
       <c r="H219" s="4" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
     </row>
     <row r="220" spans="1:8">
@@ -32323,13 +32267,13 @@
         <v>8</v>
       </c>
       <c r="B220" s="2" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="C220" s="2">
         <v>0</v>
       </c>
       <c r="D220" s="2" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="E220" s="2" t="s">
         <v>11</v>
@@ -32338,10 +32282,10 @@
         <v>12</v>
       </c>
       <c r="G220" s="3" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="H220" s="4" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
     </row>
     <row r="221" spans="1:8">
@@ -32349,13 +32293,13 @@
         <v>8</v>
       </c>
       <c r="B221" s="2" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="C221" s="2">
         <v>0</v>
       </c>
       <c r="D221" s="2" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="E221" s="2" t="s">
         <v>11</v>
@@ -32364,10 +32308,10 @@
         <v>12</v>
       </c>
       <c r="G221" s="3" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="H221" s="4" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
     </row>
     <row r="222" spans="1:8">
@@ -32375,13 +32319,13 @@
         <v>8</v>
       </c>
       <c r="B222" s="2" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="C222" s="2">
         <v>0</v>
       </c>
       <c r="D222" s="2" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="E222" s="2" t="s">
         <v>11</v>
@@ -32390,10 +32334,10 @@
         <v>12</v>
       </c>
       <c r="G222" s="3" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="H222" s="4" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
     </row>
     <row r="223" spans="1:8">
@@ -32401,13 +32345,13 @@
         <v>8</v>
       </c>
       <c r="B223" s="2" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="C223" s="2">
         <v>0</v>
       </c>
       <c r="D223" s="2" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="E223" s="2" t="s">
         <v>11</v>
@@ -32416,10 +32360,10 @@
         <v>12</v>
       </c>
       <c r="G223" s="3" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="H223" s="4" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
     </row>
     <row r="224" spans="1:8">
@@ -32427,13 +32371,13 @@
         <v>8</v>
       </c>
       <c r="B224" s="2" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="C224" s="2">
         <v>0</v>
       </c>
       <c r="D224" s="2" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="E224" s="2" t="s">
         <v>11</v>
@@ -32442,10 +32386,10 @@
         <v>12</v>
       </c>
       <c r="G224" s="3" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="H224" s="4" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
     </row>
     <row r="225" spans="1:8" ht="28.8">
@@ -32453,13 +32397,13 @@
         <v>8</v>
       </c>
       <c r="B225" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C225" s="2">
         <v>0</v>
       </c>
       <c r="D225" s="2" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="E225" s="2" t="s">
         <v>11</v>
@@ -32468,10 +32412,10 @@
         <v>12</v>
       </c>
       <c r="G225" s="3" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="H225" s="4" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
     </row>
     <row r="226" spans="1:8" ht="28.8">
@@ -32479,13 +32423,13 @@
         <v>8</v>
       </c>
       <c r="B226" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C226" s="2">
         <v>1</v>
       </c>
       <c r="D226" s="2" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="E226" s="2" t="s">
         <v>11</v>
@@ -32494,10 +32438,10 @@
         <v>12</v>
       </c>
       <c r="G226" s="3" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="H226" s="4" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
     </row>
     <row r="227" spans="1:8">
@@ -32505,13 +32449,13 @@
         <v>8</v>
       </c>
       <c r="B227" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C227" s="2">
         <v>2</v>
       </c>
       <c r="D227" s="2" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="E227" s="2" t="s">
         <v>11</v>
@@ -32520,10 +32464,10 @@
         <v>12</v>
       </c>
       <c r="G227" s="3" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="H227" s="4" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
     </row>
     <row r="228" spans="1:8" ht="100.8">
@@ -32531,13 +32475,13 @@
         <v>8</v>
       </c>
       <c r="B228" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C228" s="2">
         <v>3</v>
       </c>
       <c r="D228" s="2" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="E228" s="2" t="s">
         <v>11</v>
@@ -32546,10 +32490,10 @@
         <v>12</v>
       </c>
       <c r="G228" s="3" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="H228" s="3" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
     </row>
     <row r="229" spans="1:8" ht="187.2">
@@ -32557,13 +32501,13 @@
         <v>8</v>
       </c>
       <c r="B229" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C229" s="2">
         <v>4</v>
       </c>
       <c r="D229" s="2" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="E229" s="2" t="s">
         <v>11</v>
@@ -32572,10 +32516,10 @@
         <v>12</v>
       </c>
       <c r="G229" s="3" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="H229" s="3" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
     </row>
     <row r="230" spans="1:8" ht="100.8">
@@ -32583,13 +32527,13 @@
         <v>8</v>
       </c>
       <c r="B230" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C230" s="2">
         <v>5</v>
       </c>
       <c r="D230" s="2" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="E230" s="2" t="s">
         <v>11</v>
@@ -32598,10 +32542,10 @@
         <v>12</v>
       </c>
       <c r="G230" s="3" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="H230" s="3" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
     </row>
     <row r="231" spans="1:8" ht="100.8">
@@ -32609,13 +32553,13 @@
         <v>8</v>
       </c>
       <c r="B231" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C231" s="2">
         <v>6</v>
       </c>
       <c r="D231" s="2" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="E231" s="2" t="s">
         <v>11</v>
@@ -32624,10 +32568,10 @@
         <v>12</v>
       </c>
       <c r="G231" s="3" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="H231" s="3" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
     </row>
     <row r="232" spans="1:8" ht="43.2">
@@ -32635,13 +32579,13 @@
         <v>8</v>
       </c>
       <c r="B232" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C232" s="2">
         <v>7</v>
       </c>
       <c r="D232" s="2" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="E232" s="2" t="s">
         <v>11</v>
@@ -32650,10 +32594,10 @@
         <v>12</v>
       </c>
       <c r="G232" s="3" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="H232" s="3" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
     </row>
     <row r="233" spans="1:8" ht="100.8">
@@ -32661,13 +32605,13 @@
         <v>8</v>
       </c>
       <c r="B233" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C233" s="2">
         <v>8</v>
       </c>
       <c r="D233" s="2" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="E233" s="2" t="s">
         <v>11</v>
@@ -32676,10 +32620,10 @@
         <v>12</v>
       </c>
       <c r="G233" s="3" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="H233" s="3" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
     </row>
     <row r="234" spans="1:8" ht="43.2">
@@ -32687,13 +32631,13 @@
         <v>8</v>
       </c>
       <c r="B234" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C234" s="2">
         <v>9</v>
       </c>
       <c r="D234" s="2" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="E234" s="2" t="s">
         <v>11</v>
@@ -32702,10 +32646,10 @@
         <v>12</v>
       </c>
       <c r="G234" s="3" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="H234" s="3" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
     </row>
     <row r="235" spans="1:8" ht="409.6">
@@ -32713,13 +32657,13 @@
         <v>8</v>
       </c>
       <c r="B235" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C235" s="2">
         <v>10</v>
       </c>
       <c r="D235" s="2" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="E235" s="2" t="s">
         <v>11</v>
@@ -32728,10 +32672,10 @@
         <v>12</v>
       </c>
       <c r="G235" s="3" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="H235" s="3" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
     </row>
     <row r="236" spans="1:8" ht="43.2">
@@ -32739,13 +32683,13 @@
         <v>8</v>
       </c>
       <c r="B236" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C236" s="2">
         <v>11</v>
       </c>
       <c r="D236" s="2" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="E236" s="2" t="s">
         <v>11</v>
@@ -32754,10 +32698,10 @@
         <v>12</v>
       </c>
       <c r="G236" s="3" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="H236" s="3" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="237" spans="1:8" ht="43.2">
@@ -32765,13 +32709,13 @@
         <v>8</v>
       </c>
       <c r="B237" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C237" s="2">
         <v>12</v>
       </c>
       <c r="D237" s="2" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="E237" s="2" t="s">
         <v>11</v>
@@ -32780,10 +32724,10 @@
         <v>12</v>
       </c>
       <c r="G237" s="3" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="H237" s="3" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
     </row>
     <row r="238" spans="1:8" ht="115.2">
@@ -32791,13 +32735,13 @@
         <v>8</v>
       </c>
       <c r="B238" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C238" s="2">
         <v>13</v>
       </c>
       <c r="D238" s="2" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="E238" s="2" t="s">
         <v>11</v>
@@ -32806,10 +32750,10 @@
         <v>12</v>
       </c>
       <c r="G238" s="3" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="H238" s="3" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
     </row>
     <row r="239" spans="1:8" ht="43.2">
@@ -32817,13 +32761,13 @@
         <v>8</v>
       </c>
       <c r="B239" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C239" s="2">
         <v>14</v>
       </c>
       <c r="D239" s="2" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="E239" s="2" t="s">
         <v>11</v>
@@ -32832,10 +32776,10 @@
         <v>12</v>
       </c>
       <c r="G239" s="3" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="H239" s="3" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
     </row>
     <row r="240" spans="1:8" ht="43.2">
@@ -32843,13 +32787,13 @@
         <v>8</v>
       </c>
       <c r="B240" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C240" s="2">
         <v>15</v>
       </c>
       <c r="D240" s="2" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="E240" s="2" t="s">
         <v>11</v>
@@ -32858,10 +32802,10 @@
         <v>12</v>
       </c>
       <c r="G240" s="3" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="H240" s="3" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
     </row>
     <row r="241" spans="1:8" ht="115.2">
@@ -32869,13 +32813,13 @@
         <v>8</v>
       </c>
       <c r="B241" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C241" s="2">
         <v>16</v>
       </c>
       <c r="D241" s="2" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="E241" s="2" t="s">
         <v>11</v>
@@ -32884,10 +32828,10 @@
         <v>12</v>
       </c>
       <c r="G241" s="3" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="H241" s="3" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
     </row>
     <row r="242" spans="1:8" ht="129.6">
@@ -32895,13 +32839,13 @@
         <v>8</v>
       </c>
       <c r="B242" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C242" s="2">
         <v>17</v>
       </c>
       <c r="D242" s="2" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="E242" s="2" t="s">
         <v>11</v>
@@ -32910,10 +32854,10 @@
         <v>12</v>
       </c>
       <c r="G242" s="3" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="H242" s="3" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
     </row>
     <row r="243" spans="1:8" ht="129.6">
@@ -32921,13 +32865,13 @@
         <v>8</v>
       </c>
       <c r="B243" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C243" s="2">
         <v>18</v>
       </c>
       <c r="D243" s="2" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="E243" s="2" t="s">
         <v>11</v>
@@ -32936,10 +32880,10 @@
         <v>12</v>
       </c>
       <c r="G243" s="3" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="H243" s="3" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
     </row>
     <row r="244" spans="1:8" ht="100.8">
@@ -32947,13 +32891,13 @@
         <v>8</v>
       </c>
       <c r="B244" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C244" s="2">
         <v>19</v>
       </c>
       <c r="D244" s="2" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="E244" s="2" t="s">
         <v>11</v>
@@ -32962,10 +32906,10 @@
         <v>12</v>
       </c>
       <c r="G244" s="3" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="H244" s="3" t="s">
-        <v>710</v>
+        <v>708</v>
       </c>
     </row>
     <row r="245" spans="1:8" ht="86.4">
@@ -32973,13 +32917,13 @@
         <v>8</v>
       </c>
       <c r="B245" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C245" s="2">
         <v>20</v>
       </c>
       <c r="D245" s="2" t="s">
-        <v>711</v>
+        <v>709</v>
       </c>
       <c r="E245" s="2" t="s">
         <v>11</v>
@@ -32988,10 +32932,10 @@
         <v>12</v>
       </c>
       <c r="G245" s="3" t="s">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="H245" s="3" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
     </row>
     <row r="246" spans="1:8" ht="216">
@@ -32999,13 +32943,13 @@
         <v>8</v>
       </c>
       <c r="B246" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C246" s="2">
         <v>21</v>
       </c>
       <c r="D246" s="2" t="s">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="E246" s="2" t="s">
         <v>11</v>
@@ -33014,10 +32958,10 @@
         <v>12</v>
       </c>
       <c r="G246" s="3" t="s">
-        <v>715</v>
+        <v>713</v>
       </c>
       <c r="H246" s="3" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
     </row>
     <row r="247" spans="1:8" ht="100.8">
@@ -33025,13 +32969,13 @@
         <v>8</v>
       </c>
       <c r="B247" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C247" s="2">
         <v>22</v>
       </c>
       <c r="D247" s="2" t="s">
-        <v>717</v>
+        <v>715</v>
       </c>
       <c r="E247" s="2" t="s">
         <v>11</v>
@@ -33040,10 +32984,10 @@
         <v>12</v>
       </c>
       <c r="G247" s="3" t="s">
-        <v>718</v>
+        <v>716</v>
       </c>
       <c r="H247" s="3" t="s">
-        <v>719</v>
+        <v>717</v>
       </c>
     </row>
     <row r="248" spans="1:8" ht="187.2">
@@ -33051,13 +32995,13 @@
         <v>8</v>
       </c>
       <c r="B248" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C248" s="2">
         <v>23</v>
       </c>
       <c r="D248" s="2" t="s">
-        <v>720</v>
+        <v>718</v>
       </c>
       <c r="E248" s="2" t="s">
         <v>11</v>
@@ -33066,10 +33010,10 @@
         <v>12</v>
       </c>
       <c r="G248" s="3" t="s">
-        <v>721</v>
+        <v>719</v>
       </c>
       <c r="H248" s="3" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
     </row>
     <row r="249" spans="1:8" ht="28.8">
@@ -33077,13 +33021,13 @@
         <v>8</v>
       </c>
       <c r="B249" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C249" s="2">
         <v>24</v>
       </c>
       <c r="D249" s="2" t="s">
-        <v>723</v>
+        <v>721</v>
       </c>
       <c r="E249" s="2" t="s">
         <v>11</v>
@@ -33092,10 +33036,10 @@
         <v>12</v>
       </c>
       <c r="G249" s="3" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="H249" s="4" t="s">
-        <v>725</v>
+        <v>723</v>
       </c>
     </row>
     <row r="250" spans="1:8" ht="43.2">
@@ -33103,13 +33047,13 @@
         <v>8</v>
       </c>
       <c r="B250" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C250" s="2">
         <v>25</v>
       </c>
       <c r="D250" s="2" t="s">
-        <v>726</v>
+        <v>724</v>
       </c>
       <c r="E250" s="2" t="s">
         <v>11</v>
@@ -33118,10 +33062,10 @@
         <v>12</v>
       </c>
       <c r="G250" s="3" t="s">
-        <v>727</v>
+        <v>725</v>
       </c>
       <c r="H250" s="3" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
     </row>
     <row r="251" spans="1:8" ht="43.2">
@@ -33129,13 +33073,13 @@
         <v>8</v>
       </c>
       <c r="B251" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C251" s="2">
         <v>26</v>
       </c>
       <c r="D251" s="2" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="E251" s="2" t="s">
         <v>11</v>
@@ -33144,10 +33088,10 @@
         <v>12</v>
       </c>
       <c r="G251" s="3" t="s">
-        <v>730</v>
+        <v>728</v>
       </c>
       <c r="H251" s="3" t="s">
-        <v>731</v>
+        <v>729</v>
       </c>
     </row>
     <row r="252" spans="1:8" ht="43.2">
@@ -33155,13 +33099,13 @@
         <v>8</v>
       </c>
       <c r="B252" s="2" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="C252" s="2">
         <v>27</v>
       </c>
       <c r="D252" s="2" t="s">
-        <v>732</v>
+        <v>730</v>
       </c>
       <c r="E252" s="2" t="s">
         <v>11</v>
@@ -33170,10 +33114,10 @@
         <v>12</v>
       </c>
       <c r="G252" s="3" t="s">
-        <v>733</v>
+        <v>731</v>
       </c>
       <c r="H252" s="3" t="s">
-        <v>734</v>
+        <v>732</v>
       </c>
     </row>
     <row r="253" spans="1:8">
@@ -33181,13 +33125,13 @@
         <v>8</v>
       </c>
       <c r="B253" s="2" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="C253" s="2">
         <v>0</v>
       </c>
       <c r="D253" s="2" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
       <c r="E253" s="2" t="s">
         <v>11</v>
@@ -33196,10 +33140,10 @@
         <v>12</v>
       </c>
       <c r="G253" s="3" t="s">
-        <v>737</v>
+        <v>735</v>
       </c>
       <c r="H253" s="4" t="s">
-        <v>738</v>
+        <v>736</v>
       </c>
     </row>
     <row r="254" spans="1:8" ht="100.8">
@@ -33207,13 +33151,13 @@
         <v>8</v>
       </c>
       <c r="B254" s="2" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="C254" s="2">
         <v>2</v>
       </c>
       <c r="D254" s="2" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="E254" s="2" t="s">
         <v>11</v>
@@ -33222,10 +33166,10 @@
         <v>12</v>
       </c>
       <c r="G254" s="3" t="s">
-        <v>740</v>
+        <v>738</v>
       </c>
       <c r="H254" s="3" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
     </row>
     <row r="255" spans="1:8">
@@ -33233,13 +33177,13 @@
         <v>8</v>
       </c>
       <c r="B255" s="2" t="s">
-        <v>742</v>
+        <v>740</v>
       </c>
       <c r="C255" s="2">
         <v>0</v>
       </c>
       <c r="D255" s="2" t="s">
-        <v>743</v>
+        <v>741</v>
       </c>
       <c r="E255" s="2" t="s">
         <v>11</v>
@@ -33248,10 +33192,10 @@
         <v>12</v>
       </c>
       <c r="G255" s="3" t="s">
-        <v>744</v>
+        <v>742</v>
       </c>
       <c r="H255" s="4" t="s">
-        <v>745</v>
+        <v>743</v>
       </c>
     </row>
     <row r="256" spans="1:8">
@@ -33259,13 +33203,13 @@
         <v>8</v>
       </c>
       <c r="B256" s="2" t="s">
-        <v>746</v>
+        <v>744</v>
       </c>
       <c r="C256" s="2">
         <v>0</v>
       </c>
       <c r="D256" s="2" t="s">
-        <v>747</v>
+        <v>745</v>
       </c>
       <c r="E256" s="2" t="s">
         <v>11</v>
@@ -33274,10 +33218,10 @@
         <v>12</v>
       </c>
       <c r="G256" s="3" t="s">
-        <v>748</v>
+        <v>746</v>
       </c>
       <c r="H256" s="4" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
     </row>
     <row r="257" spans="1:8" ht="28.8">
@@ -33285,13 +33229,13 @@
         <v>8</v>
       </c>
       <c r="B257" s="2" t="s">
-        <v>750</v>
+        <v>748</v>
       </c>
       <c r="C257" s="2">
         <v>0</v>
       </c>
       <c r="D257" s="2" t="s">
-        <v>751</v>
+        <v>749</v>
       </c>
       <c r="E257" s="2" t="s">
         <v>11</v>
@@ -33300,10 +33244,10 @@
         <v>12</v>
       </c>
       <c r="G257" s="3" t="s">
-        <v>752</v>
+        <v>750</v>
       </c>
       <c r="H257" s="3" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
     </row>
     <row r="258" spans="1:8" ht="43.2">
@@ -33311,13 +33255,13 @@
         <v>8</v>
       </c>
       <c r="B258" s="2" t="s">
-        <v>750</v>
+        <v>748</v>
       </c>
       <c r="C258" s="2">
         <v>1</v>
       </c>
       <c r="D258" s="2" t="s">
-        <v>754</v>
+        <v>752</v>
       </c>
       <c r="E258" s="2" t="s">
         <v>11</v>
@@ -33326,10 +33270,10 @@
         <v>12</v>
       </c>
       <c r="G258" s="3" t="s">
-        <v>755</v>
+        <v>753</v>
       </c>
       <c r="H258" s="3" t="s">
-        <v>756</v>
+        <v>754</v>
       </c>
     </row>
     <row r="259" spans="1:8" ht="100.8">
@@ -33337,13 +33281,13 @@
         <v>8</v>
       </c>
       <c r="B259" s="2" t="s">
-        <v>750</v>
+        <v>748</v>
       </c>
       <c r="C259" s="2">
         <v>2</v>
       </c>
       <c r="D259" s="2" t="s">
-        <v>757</v>
+        <v>755</v>
       </c>
       <c r="E259" s="2" t="s">
         <v>11</v>
@@ -33352,10 +33296,10 @@
         <v>12</v>
       </c>
       <c r="G259" s="3" t="s">
-        <v>758</v>
+        <v>756</v>
       </c>
       <c r="H259" s="3" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
     </row>
     <row r="260" spans="1:8" ht="43.2">
@@ -33363,13 +33307,13 @@
         <v>8</v>
       </c>
       <c r="B260" s="2" t="s">
-        <v>750</v>
+        <v>748</v>
       </c>
       <c r="C260" s="2">
         <v>3</v>
       </c>
       <c r="D260" s="2" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
       <c r="E260" s="2" t="s">
         <v>11</v>
@@ -33378,10 +33322,10 @@
         <v>12</v>
       </c>
       <c r="G260" s="3" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="H260" s="3" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
     </row>
     <row r="261" spans="1:8">
@@ -33389,13 +33333,13 @@
         <v>8</v>
       </c>
       <c r="B261" s="2" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
       <c r="C261" s="2">
         <v>0</v>
       </c>
       <c r="D261" s="2" t="s">
-        <v>764</v>
+        <v>762</v>
       </c>
       <c r="E261" s="2" t="s">
         <v>11</v>
@@ -33404,10 +33348,10 @@
         <v>12</v>
       </c>
       <c r="G261" s="3" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
       <c r="H261" s="4" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
     </row>
     <row r="262" spans="1:8">
@@ -33415,13 +33359,13 @@
         <v>8</v>
       </c>
       <c r="B262" s="2" t="s">
-        <v>767</v>
+        <v>765</v>
       </c>
       <c r="C262" s="2">
         <v>0</v>
       </c>
       <c r="D262" s="2" t="s">
-        <v>768</v>
+        <v>766</v>
       </c>
       <c r="E262" s="2" t="s">
         <v>11</v>
@@ -33430,10 +33374,10 @@
         <v>12</v>
       </c>
       <c r="G262" s="3" t="s">
-        <v>769</v>
+        <v>767</v>
       </c>
       <c r="H262" s="4" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
     </row>
     <row r="263" spans="1:8">
@@ -33441,13 +33385,13 @@
         <v>8</v>
       </c>
       <c r="B263" s="2" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="C263" s="2">
         <v>0</v>
       </c>
       <c r="D263" s="2" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
       <c r="E263" s="2" t="s">
         <v>11</v>
@@ -33456,10 +33400,10 @@
         <v>12</v>
       </c>
       <c r="G263" s="3" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="H263" s="4" t="s">
-        <v>774</v>
+        <v>772</v>
       </c>
     </row>
     <row r="264" spans="1:8">
@@ -33467,13 +33411,13 @@
         <v>8</v>
       </c>
       <c r="B264" s="2" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="C264" s="2">
         <v>1</v>
       </c>
       <c r="D264" s="2" t="s">
-        <v>775</v>
+        <v>773</v>
       </c>
       <c r="E264" s="2" t="s">
         <v>11</v>
@@ -33482,10 +33426,10 @@
         <v>12</v>
       </c>
       <c r="G264" s="3" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="H264" s="4" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
     </row>
     <row r="265" spans="1:8" ht="28.8">
@@ -33493,13 +33437,13 @@
         <v>8</v>
       </c>
       <c r="B265" s="2" t="s">
-        <v>778</v>
+        <v>776</v>
       </c>
       <c r="C265" s="2">
         <v>0</v>
       </c>
       <c r="D265" s="2" t="s">
-        <v>779</v>
+        <v>777</v>
       </c>
       <c r="E265" s="2" t="s">
         <v>11</v>
@@ -33508,10 +33452,10 @@
         <v>12</v>
       </c>
       <c r="G265" s="3" t="s">
-        <v>780</v>
+        <v>778</v>
       </c>
       <c r="H265" s="4" t="s">
-        <v>781</v>
+        <v>779</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
additional updates before final internal review
</commit_message>
<xml_diff>
--- a/docassemble/PowerOfAttorneyProperty/data/sources/poa_property_es.xlsx
+++ b/docassemble/PowerOfAttorneyProperty/data/sources/poa_property_es.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\local-DA-easyforms-dev\sources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FADC3D69-E4A2-4306-ABAE-0B8DFC2924BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD53EF1A-201E-4428-8367-63AE692310AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38625" yWindow="-3330" windowWidth="35685" windowHeight="16530" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-34920" yWindow="-525" windowWidth="25725" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>